<commit_message>
feat: add forward-looking macro views and slide text appendix
- Section 10: current macro regime assessment (Overheating, tariff shock,
  Fed hold), 2026 midterm scenario matrix, per-position analyst views
  for all 16 holdings with macro/political overlay and conviction ratings
- Section 10d: portfolio construction recommendations for incoming managers
- Section 11: verbatim presentation text for slides 13, 14, 15, 17-18, 20
  including reasoning column fill for all positions in the implications slides
- Re-render to PDF (55 chunks, clean output)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/llb_transactions.xlsx
+++ b/llb_transactions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wu-my.sharepoint.com/personal/h12420126_s_wu_ac_at/Documents/00_WU/02_PMP/Manager_year/last_manager_presenation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_4A6528E9373E6C93A62BB8B3B6DD66E13733FCCD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3DE5628-7066-8C4C-86F0-8427F4280E04}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_4A6528E9373E6C93A62BB8B3B6DD66E13733FCCD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C11872E3-077F-DA4A-A5C7-D5E08E3EB724}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -345,10 +345,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
-    <numFmt numFmtId="166" formatCode="dd\.mm\.yyyy"/>
-    <numFmt numFmtId="191" formatCode="#,##0.000000"/>
-    <numFmt numFmtId="198" formatCode="#,##0\ [$Piece]"/>
-    <numFmt numFmtId="212" formatCode="#,##0\ [$Units]"/>
+    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
+    <numFmt numFmtId="165" formatCode="#,##0.000000"/>
+    <numFmt numFmtId="166" formatCode="#,##0\ [$Piece]"/>
+    <numFmt numFmtId="167" formatCode="#,##0\ [$Units]"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -389,10 +389,10 @@
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="191" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="198" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="212" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -408,6 +408,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -713,7 +717,7 @@
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="21" customWidth="1"/>
     <col min="5" max="5" width="24" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
+    <col min="6" max="6" width="51.33203125" customWidth="1"/>
     <col min="7" max="7" width="28" customWidth="1"/>
     <col min="8" max="8" width="18" customWidth="1"/>
     <col min="9" max="11" width="28" customWidth="1"/>

</xml_diff>